<commit_message>
feat: pension benefits and rent income
- Add feature to include pension survivor benefits
- Add feature to account for rent and trust income separately for NIIT
- Update all docs
- Audit rate models and fix few discrepancies
</commit_message>
<xml_diff>
--- a/examples/HFP_alex+jamie.xlsx
+++ b/examples/HFP_alex+jamie.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J36"/>
+  <dimension ref="A1:K36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,35 +449,40 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>net inv</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>taxable ctrb</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>401k ctrb</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Roth 401k ctrb</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>IRA ctrb</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Roth IRA ctrb</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Roth conv</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>big-ticket items</t>
         </is>
@@ -491,15 +496,18 @@
       <c r="C2" t="n">
         <v>0</v>
       </c>
-      <c r="D2" t="inlineStr"/>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
-      <c r="G2" t="n">
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="n">
         <v>6500</v>
       </c>
-      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -509,15 +517,18 @@
       <c r="C3" t="n">
         <v>0</v>
       </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
-      <c r="G3" t="n">
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="n">
         <v>6500</v>
       </c>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -527,15 +538,18 @@
       <c r="C4" t="n">
         <v>0</v>
       </c>
-      <c r="D4" t="inlineStr"/>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
-      <c r="G4" t="n">
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="n">
         <v>7000</v>
       </c>
-      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -545,15 +559,18 @@
       <c r="C5" t="n">
         <v>0</v>
       </c>
-      <c r="D5" t="inlineStr"/>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
-      <c r="G5" t="n">
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="n">
         <v>7000</v>
       </c>
-      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -563,17 +580,20 @@
       <c r="C6" t="n">
         <v>0</v>
       </c>
-      <c r="D6" t="inlineStr"/>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
-      <c r="G6" t="n">
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="n">
         <v>7000</v>
       </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="n">
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="n">
         <v>20000</v>
       </c>
-      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -585,15 +605,18 @@
       <c r="C7" t="n">
         <v>0</v>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="n">
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="n">
         <v>15000</v>
       </c>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -605,15 +628,18 @@
       <c r="C8" t="n">
         <v>0</v>
       </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="n">
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="n">
         <v>15000</v>
       </c>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -625,15 +651,18 @@
       <c r="C9" t="n">
         <v>0</v>
       </c>
-      <c r="D9" t="inlineStr"/>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" t="n">
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="n">
         <v>50000</v>
       </c>
-      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -643,15 +672,18 @@
       <c r="C10" t="n">
         <v>0</v>
       </c>
-      <c r="D10" t="inlineStr"/>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
-      <c r="I10" t="n">
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="n">
         <v>50000</v>
       </c>
-      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -661,13 +693,16 @@
       <c r="C11" t="n">
         <v>0</v>
       </c>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -677,13 +712,16 @@
       <c r="C12" t="n">
         <v>0</v>
       </c>
-      <c r="D12" t="inlineStr"/>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -693,13 +731,16 @@
       <c r="C13" t="n">
         <v>0</v>
       </c>
-      <c r="D13" t="inlineStr"/>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -709,13 +750,16 @@
       <c r="C14" t="n">
         <v>0</v>
       </c>
-      <c r="D14" t="inlineStr"/>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -725,13 +769,16 @@
       <c r="C15" t="n">
         <v>0</v>
       </c>
-      <c r="D15" t="inlineStr"/>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -741,13 +788,16 @@
       <c r="C16" t="n">
         <v>0</v>
       </c>
-      <c r="D16" t="inlineStr"/>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -757,13 +807,16 @@
       <c r="C17" t="n">
         <v>0</v>
       </c>
-      <c r="D17" t="inlineStr"/>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -773,13 +826,16 @@
       <c r="C18" t="n">
         <v>0</v>
       </c>
-      <c r="D18" t="inlineStr"/>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -789,13 +845,16 @@
       <c r="C19" t="n">
         <v>0</v>
       </c>
-      <c r="D19" t="inlineStr"/>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -805,13 +864,16 @@
       <c r="C20" t="n">
         <v>0</v>
       </c>
-      <c r="D20" t="inlineStr"/>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -821,13 +883,16 @@
       <c r="C21" t="n">
         <v>0</v>
       </c>
-      <c r="D21" t="inlineStr"/>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -837,13 +902,16 @@
       <c r="C22" t="n">
         <v>0</v>
       </c>
-      <c r="D22" t="inlineStr"/>
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -853,13 +921,16 @@
       <c r="C23" t="n">
         <v>0</v>
       </c>
-      <c r="D23" t="inlineStr"/>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -869,13 +940,16 @@
       <c r="C24" t="n">
         <v>0</v>
       </c>
-      <c r="D24" t="inlineStr"/>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -885,13 +959,16 @@
       <c r="C25" t="n">
         <v>0</v>
       </c>
-      <c r="D25" t="inlineStr"/>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -901,13 +978,16 @@
       <c r="C26" t="n">
         <v>0</v>
       </c>
-      <c r="D26" t="inlineStr"/>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -917,13 +997,16 @@
       <c r="C27" t="n">
         <v>0</v>
       </c>
-      <c r="D27" t="inlineStr"/>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -933,13 +1016,16 @@
       <c r="C28" t="n">
         <v>0</v>
       </c>
-      <c r="D28" t="inlineStr"/>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -949,13 +1035,16 @@
       <c r="C29" t="n">
         <v>0</v>
       </c>
-      <c r="D29" t="inlineStr"/>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -965,13 +1054,16 @@
       <c r="C30" t="n">
         <v>0</v>
       </c>
-      <c r="D30" t="inlineStr"/>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -981,13 +1073,16 @@
       <c r="C31" t="n">
         <v>0</v>
       </c>
-      <c r="D31" t="inlineStr"/>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -997,13 +1092,16 @@
       <c r="C32" t="n">
         <v>0</v>
       </c>
-      <c r="D32" t="inlineStr"/>
+      <c r="D32" t="n">
+        <v>0</v>
+      </c>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1013,13 +1111,16 @@
       <c r="C33" t="n">
         <v>0</v>
       </c>
-      <c r="D33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>0</v>
+      </c>
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1029,13 +1130,16 @@
       <c r="C34" t="n">
         <v>0</v>
       </c>
-      <c r="D34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>0</v>
+      </c>
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1045,13 +1149,16 @@
       <c r="C35" t="n">
         <v>0</v>
       </c>
-      <c r="D35" t="inlineStr"/>
+      <c r="D35" t="n">
+        <v>0</v>
+      </c>
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1061,13 +1168,16 @@
       <c r="C36" t="n">
         <v>0</v>
       </c>
-      <c r="D36" t="inlineStr"/>
+      <c r="D36" t="n">
+        <v>0</v>
+      </c>
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1080,7 +1190,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J39"/>
+  <dimension ref="A1:K39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1101,35 +1211,40 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>net inv</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>taxable ctrb</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>401k ctrb</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Roth 401k ctrb</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>IRA ctrb</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Roth IRA ctrb</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Roth conv</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>big-ticket items</t>
         </is>
@@ -1143,15 +1258,18 @@
       <c r="C2" t="n">
         <v>0</v>
       </c>
-      <c r="D2" t="inlineStr"/>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" t="n">
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="n">
         <v>4000</v>
       </c>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -1161,15 +1279,18 @@
       <c r="C3" t="n">
         <v>0</v>
       </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" t="n">
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="n">
         <v>4000</v>
       </c>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -1179,15 +1300,18 @@
       <c r="C4" t="n">
         <v>0</v>
       </c>
-      <c r="D4" t="inlineStr"/>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
-      <c r="H4" t="n">
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="n">
         <v>4000</v>
       </c>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1197,15 +1321,18 @@
       <c r="C5" t="n">
         <v>0</v>
       </c>
-      <c r="D5" t="inlineStr"/>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
-      <c r="I5" t="n">
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="n">
         <v>12000</v>
       </c>
-      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1215,15 +1342,18 @@
       <c r="C6" t="n">
         <v>0</v>
       </c>
-      <c r="D6" t="inlineStr"/>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" t="n">
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="n">
         <v>5000</v>
       </c>
-      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1235,13 +1365,16 @@
       <c r="C7" t="n">
         <v>0</v>
       </c>
-      <c r="D7" t="inlineStr"/>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1253,13 +1386,16 @@
       <c r="C8" t="n">
         <v>0</v>
       </c>
-      <c r="D8" t="inlineStr"/>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1271,13 +1407,16 @@
       <c r="C9" t="n">
         <v>0</v>
       </c>
-      <c r="D9" t="inlineStr"/>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1287,13 +1426,16 @@
       <c r="C10" t="n">
         <v>0</v>
       </c>
-      <c r="D10" t="inlineStr"/>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1303,13 +1445,16 @@
       <c r="C11" t="n">
         <v>0</v>
       </c>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1319,13 +1464,16 @@
       <c r="C12" t="n">
         <v>0</v>
       </c>
-      <c r="D12" t="inlineStr"/>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1335,13 +1483,16 @@
       <c r="C13" t="n">
         <v>0</v>
       </c>
-      <c r="D13" t="inlineStr"/>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1351,13 +1502,16 @@
       <c r="C14" t="n">
         <v>0</v>
       </c>
-      <c r="D14" t="inlineStr"/>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1367,13 +1521,16 @@
       <c r="C15" t="n">
         <v>0</v>
       </c>
-      <c r="D15" t="inlineStr"/>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1383,13 +1540,16 @@
       <c r="C16" t="n">
         <v>0</v>
       </c>
-      <c r="D16" t="inlineStr"/>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1399,13 +1559,16 @@
       <c r="C17" t="n">
         <v>0</v>
       </c>
-      <c r="D17" t="inlineStr"/>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1415,13 +1578,16 @@
       <c r="C18" t="n">
         <v>0</v>
       </c>
-      <c r="D18" t="inlineStr"/>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1431,13 +1597,16 @@
       <c r="C19" t="n">
         <v>0</v>
       </c>
-      <c r="D19" t="inlineStr"/>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1447,13 +1616,16 @@
       <c r="C20" t="n">
         <v>0</v>
       </c>
-      <c r="D20" t="inlineStr"/>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1463,13 +1635,16 @@
       <c r="C21" t="n">
         <v>0</v>
       </c>
-      <c r="D21" t="inlineStr"/>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1479,13 +1654,16 @@
       <c r="C22" t="n">
         <v>0</v>
       </c>
-      <c r="D22" t="inlineStr"/>
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1495,13 +1673,16 @@
       <c r="C23" t="n">
         <v>0</v>
       </c>
-      <c r="D23" t="inlineStr"/>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1511,13 +1692,16 @@
       <c r="C24" t="n">
         <v>0</v>
       </c>
-      <c r="D24" t="inlineStr"/>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1527,13 +1711,16 @@
       <c r="C25" t="n">
         <v>0</v>
       </c>
-      <c r="D25" t="inlineStr"/>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1543,13 +1730,16 @@
       <c r="C26" t="n">
         <v>0</v>
       </c>
-      <c r="D26" t="inlineStr"/>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1559,13 +1749,16 @@
       <c r="C27" t="n">
         <v>0</v>
       </c>
-      <c r="D27" t="inlineStr"/>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1575,13 +1768,16 @@
       <c r="C28" t="n">
         <v>0</v>
       </c>
-      <c r="D28" t="inlineStr"/>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1591,13 +1787,16 @@
       <c r="C29" t="n">
         <v>0</v>
       </c>
-      <c r="D29" t="inlineStr"/>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1607,13 +1806,16 @@
       <c r="C30" t="n">
         <v>0</v>
       </c>
-      <c r="D30" t="inlineStr"/>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1623,13 +1825,16 @@
       <c r="C31" t="n">
         <v>0</v>
       </c>
-      <c r="D31" t="inlineStr"/>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1639,13 +1844,16 @@
       <c r="C32" t="n">
         <v>0</v>
       </c>
-      <c r="D32" t="inlineStr"/>
+      <c r="D32" t="n">
+        <v>0</v>
+      </c>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1655,13 +1863,16 @@
       <c r="C33" t="n">
         <v>0</v>
       </c>
-      <c r="D33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>0</v>
+      </c>
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1671,13 +1882,16 @@
       <c r="C34" t="n">
         <v>0</v>
       </c>
-      <c r="D34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>0</v>
+      </c>
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1687,13 +1901,16 @@
       <c r="C35" t="n">
         <v>0</v>
       </c>
-      <c r="D35" t="inlineStr"/>
+      <c r="D35" t="n">
+        <v>0</v>
+      </c>
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1703,13 +1920,16 @@
       <c r="C36" t="n">
         <v>0</v>
       </c>
-      <c r="D36" t="inlineStr"/>
+      <c r="D36" t="n">
+        <v>0</v>
+      </c>
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1719,13 +1939,16 @@
       <c r="C37" t="n">
         <v>0</v>
       </c>
-      <c r="D37" t="inlineStr"/>
+      <c r="D37" t="n">
+        <v>0</v>
+      </c>
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1735,13 +1958,16 @@
       <c r="C38" t="n">
         <v>0</v>
       </c>
-      <c r="D38" t="inlineStr"/>
+      <c r="D38" t="n">
+        <v>0</v>
+      </c>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1751,13 +1977,16 @@
       <c r="C39" t="n">
         <v>0</v>
       </c>
-      <c r="D39" t="inlineStr"/>
+      <c r="D39" t="n">
+        <v>0</v>
+      </c>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: HSA version complete.
- A fourth type of savings account HSA) is now in the mix. The tax advantage of HSA
is used to pay Medicare and IRMAA premiums.
- Formulation is modified to account for withdrawals
- Contributions made through W&C table
- New tests for HSA
- Rewrite examples to use new capabilities and extend coverage
- Documentation update
</commit_message>
<xml_diff>
--- a/examples/HFP_alex+jamie.xlsx
+++ b/examples/HFP_alex+jamie.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K36"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -485,6 +485,11 @@
       <c r="K1" s="1" t="inlineStr">
         <is>
           <t>big-ticket items</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>HSA ctrb</t>
         </is>
       </c>
     </row>
@@ -508,6 +513,9 @@
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -529,6 +537,9 @@
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -550,6 +561,9 @@
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -571,6 +585,9 @@
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -594,6 +611,9 @@
         <v>20000</v>
       </c>
       <c r="K6" t="inlineStr"/>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -617,6 +637,9 @@
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
+      <c r="L7" t="n">
+        <v>4000</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -640,6 +663,9 @@
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
+      <c r="L8" t="n">
+        <v>4000</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -663,6 +689,9 @@
         <v>50000</v>
       </c>
       <c r="K9" t="inlineStr"/>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -684,6 +713,9 @@
         <v>50000</v>
       </c>
       <c r="K10" t="inlineStr"/>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -703,6 +735,9 @@
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -722,6 +757,9 @@
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -741,6 +779,9 @@
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -760,6 +801,9 @@
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
+      <c r="L14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -779,6 +823,9 @@
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -798,6 +845,9 @@
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -817,6 +867,9 @@
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -836,6 +889,9 @@
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
+      <c r="L18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -855,6 +911,9 @@
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
+      <c r="L19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -874,6 +933,9 @@
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
+      <c r="L20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -893,6 +955,9 @@
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
+      <c r="L21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -912,6 +977,9 @@
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
+      <c r="L22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -931,6 +999,9 @@
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
+      <c r="L23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -950,6 +1021,9 @@
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
+      <c r="L24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -969,6 +1043,9 @@
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
+      <c r="L25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -988,6 +1065,9 @@
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr"/>
+      <c r="L26" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1007,6 +1087,9 @@
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr"/>
+      <c r="L27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1026,6 +1109,9 @@
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr"/>
+      <c r="L28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1045,6 +1131,9 @@
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr"/>
+      <c r="L29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1064,6 +1153,9 @@
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr"/>
+      <c r="L30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1083,6 +1175,9 @@
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
+      <c r="L31" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1102,6 +1197,9 @@
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr"/>
+      <c r="L32" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1121,6 +1219,9 @@
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr"/>
+      <c r="L33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1140,6 +1241,9 @@
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr"/>
+      <c r="L34" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1159,6 +1263,9 @@
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
+      <c r="L35" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1178,6 +1285,9 @@
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
+      <c r="L36" t="n">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1190,7 +1300,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K39"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1247,6 +1357,11 @@
       <c r="K1" s="1" t="inlineStr">
         <is>
           <t>big-ticket items</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>HSA ctrb</t>
         </is>
       </c>
     </row>
@@ -1270,6 +1385,9 @@
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -1291,6 +1409,9 @@
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -1312,6 +1433,9 @@
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1333,6 +1457,9 @@
         <v>12000</v>
       </c>
       <c r="K5" t="inlineStr"/>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1354,6 +1481,9 @@
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1375,6 +1505,9 @@
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
+      <c r="L7" t="n">
+        <v>4000</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1396,6 +1529,9 @@
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
+      <c r="L8" t="n">
+        <v>4000</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1417,6 +1553,9 @@
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1436,6 +1575,9 @@
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1455,6 +1597,9 @@
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1474,6 +1619,9 @@
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1493,6 +1641,9 @@
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1512,6 +1663,9 @@
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
+      <c r="L14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1531,6 +1685,9 @@
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1550,6 +1707,9 @@
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1569,6 +1729,9 @@
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1588,6 +1751,9 @@
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
+      <c r="L18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1607,6 +1773,9 @@
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
+      <c r="L19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1626,6 +1795,9 @@
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
+      <c r="L20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1645,6 +1817,9 @@
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
+      <c r="L21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1664,6 +1839,9 @@
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
+      <c r="L22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1683,6 +1861,9 @@
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
+      <c r="L23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1702,6 +1883,9 @@
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
+      <c r="L24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1721,6 +1905,9 @@
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
+      <c r="L25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1740,6 +1927,9 @@
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr"/>
+      <c r="L26" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1759,6 +1949,9 @@
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr"/>
+      <c r="L27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1778,6 +1971,9 @@
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr"/>
+      <c r="L28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1797,6 +1993,9 @@
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr"/>
+      <c r="L29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1816,6 +2015,9 @@
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr"/>
+      <c r="L30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1835,6 +2037,9 @@
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
+      <c r="L31" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1854,6 +2059,9 @@
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr"/>
+      <c r="L32" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1873,6 +2081,9 @@
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr"/>
+      <c r="L33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1892,6 +2103,9 @@
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr"/>
+      <c r="L34" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1911,6 +2125,9 @@
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
+      <c r="L35" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1930,6 +2147,9 @@
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
+      <c r="L36" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1949,6 +2169,9 @@
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr"/>
+      <c r="L37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1968,6 +2191,9 @@
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr"/>
+      <c r="L38" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1987,6 +2213,9 @@
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr"/>
+      <c r="L39" t="n">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
[feat] Fixed assets real vs nominal rate semantics — v2026.05.24
Physical asset types (residence, real estate, collectibles, precious metals)
now use a real (inflation-adjusted) growth rate; rate=0 tracks inflation.
Financial assets (stocks, fixed annuity) remain nominal. Example HFP files
updated to set residence/real estate rates to 0. Tests and CHANGELOG updated.
</commit_message>
<xml_diff>
--- a/examples/HFP_alex+jamie.xlsx
+++ b/examples/HFP_alex+jamie.xlsx
@@ -497,22 +497,15 @@
       <c r="A2" t="n">
         <v>2021</v>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
         <v>0</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
         <v>6500</v>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="n">
         <v>0</v>
       </c>
@@ -521,22 +514,15 @@
       <c r="A3" t="n">
         <v>2022</v>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
         <v>6500</v>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="n">
         <v>0</v>
       </c>
@@ -545,22 +531,15 @@
       <c r="A4" t="n">
         <v>2023</v>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
         <v>0</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
         <v>7000</v>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
       <c r="L4" t="n">
         <v>0</v>
       </c>
@@ -578,15 +557,9 @@
       <c r="D5" t="n">
         <v>0</v>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
         <v>7000</v>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
       <c r="L5" t="n">
         <v>0</v>
       </c>
@@ -604,17 +577,12 @@
       <c r="D6" t="n">
         <v>0</v>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
         <v>7000</v>
       </c>
-      <c r="I6" t="inlineStr"/>
       <c r="J6" t="n">
         <v>20000</v>
       </c>
-      <c r="K6" t="inlineStr"/>
       <c r="L6" t="n">
         <v>0</v>
       </c>
@@ -632,15 +600,9 @@
       <c r="D7" t="n">
         <v>0</v>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
         <v>15000</v>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
       <c r="L7" t="n">
         <v>4000</v>
       </c>
@@ -658,15 +620,9 @@
       <c r="D8" t="n">
         <v>0</v>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
         <v>15000</v>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
       <c r="L8" t="n">
         <v>4000</v>
       </c>
@@ -684,15 +640,9 @@
       <c r="D9" t="n">
         <v>0</v>
       </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
       <c r="J9" t="n">
         <v>50000</v>
       </c>
-      <c r="K9" t="inlineStr"/>
       <c r="L9" t="n">
         <v>0</v>
       </c>
@@ -701,22 +651,15 @@
       <c r="A10" t="n">
         <v>2029</v>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="n">
         <v>0</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
       </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
       <c r="J10" t="n">
         <v>50000</v>
       </c>
-      <c r="K10" t="inlineStr"/>
       <c r="L10" t="n">
         <v>0</v>
       </c>
@@ -725,20 +668,12 @@
       <c r="A11" t="n">
         <v>2030</v>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="n">
         <v>0</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
       </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
       <c r="L11" t="n">
         <v>0</v>
       </c>
@@ -747,20 +682,12 @@
       <c r="A12" t="n">
         <v>2031</v>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="n">
         <v>0</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
       </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
       <c r="L12" t="n">
         <v>0</v>
       </c>
@@ -769,20 +696,12 @@
       <c r="A13" t="n">
         <v>2032</v>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="n">
         <v>0</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
       </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
       <c r="L13" t="n">
         <v>0</v>
       </c>
@@ -791,20 +710,12 @@
       <c r="A14" t="n">
         <v>2033</v>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" t="n">
         <v>0</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
       </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
       <c r="L14" t="n">
         <v>0</v>
       </c>
@@ -813,20 +724,12 @@
       <c r="A15" t="n">
         <v>2034</v>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" t="n">
         <v>0</v>
       </c>
       <c r="D15" t="n">
         <v>0</v>
       </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
       <c r="L15" t="n">
         <v>0</v>
       </c>
@@ -835,20 +738,12 @@
       <c r="A16" t="n">
         <v>2035</v>
       </c>
-      <c r="B16" t="inlineStr"/>
       <c r="C16" t="n">
         <v>0</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
       </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
       <c r="L16" t="n">
         <v>0</v>
       </c>
@@ -857,20 +752,12 @@
       <c r="A17" t="n">
         <v>2036</v>
       </c>
-      <c r="B17" t="inlineStr"/>
       <c r="C17" t="n">
         <v>0</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
       </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
       <c r="L17" t="n">
         <v>0</v>
       </c>
@@ -879,20 +766,12 @@
       <c r="A18" t="n">
         <v>2037</v>
       </c>
-      <c r="B18" t="inlineStr"/>
       <c r="C18" t="n">
         <v>0</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
       </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
       <c r="L18" t="n">
         <v>0</v>
       </c>
@@ -901,20 +780,12 @@
       <c r="A19" t="n">
         <v>2038</v>
       </c>
-      <c r="B19" t="inlineStr"/>
       <c r="C19" t="n">
         <v>0</v>
       </c>
       <c r="D19" t="n">
         <v>0</v>
       </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
       <c r="L19" t="n">
         <v>0</v>
       </c>
@@ -923,20 +794,12 @@
       <c r="A20" t="n">
         <v>2039</v>
       </c>
-      <c r="B20" t="inlineStr"/>
       <c r="C20" t="n">
         <v>0</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
       </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
       <c r="L20" t="n">
         <v>0</v>
       </c>
@@ -945,20 +808,12 @@
       <c r="A21" t="n">
         <v>2040</v>
       </c>
-      <c r="B21" t="inlineStr"/>
       <c r="C21" t="n">
         <v>0</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
       </c>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
       <c r="L21" t="n">
         <v>0</v>
       </c>
@@ -967,20 +822,12 @@
       <c r="A22" t="n">
         <v>2041</v>
       </c>
-      <c r="B22" t="inlineStr"/>
       <c r="C22" t="n">
         <v>0</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
       </c>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
       <c r="L22" t="n">
         <v>0</v>
       </c>
@@ -989,20 +836,12 @@
       <c r="A23" t="n">
         <v>2042</v>
       </c>
-      <c r="B23" t="inlineStr"/>
       <c r="C23" t="n">
         <v>0</v>
       </c>
       <c r="D23" t="n">
         <v>0</v>
       </c>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
       <c r="L23" t="n">
         <v>0</v>
       </c>
@@ -1011,20 +850,12 @@
       <c r="A24" t="n">
         <v>2043</v>
       </c>
-      <c r="B24" t="inlineStr"/>
       <c r="C24" t="n">
         <v>0</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
       </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
       <c r="L24" t="n">
         <v>0</v>
       </c>
@@ -1033,20 +864,12 @@
       <c r="A25" t="n">
         <v>2044</v>
       </c>
-      <c r="B25" t="inlineStr"/>
       <c r="C25" t="n">
         <v>0</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
       </c>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
       <c r="L25" t="n">
         <v>0</v>
       </c>
@@ -1055,20 +878,12 @@
       <c r="A26" t="n">
         <v>2045</v>
       </c>
-      <c r="B26" t="inlineStr"/>
       <c r="C26" t="n">
         <v>0</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
       </c>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
       <c r="L26" t="n">
         <v>0</v>
       </c>
@@ -1077,20 +892,12 @@
       <c r="A27" t="n">
         <v>2046</v>
       </c>
-      <c r="B27" t="inlineStr"/>
       <c r="C27" t="n">
         <v>0</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
       </c>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
       <c r="L27" t="n">
         <v>0</v>
       </c>
@@ -1099,20 +906,12 @@
       <c r="A28" t="n">
         <v>2047</v>
       </c>
-      <c r="B28" t="inlineStr"/>
       <c r="C28" t="n">
         <v>0</v>
       </c>
       <c r="D28" t="n">
         <v>0</v>
       </c>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
       <c r="L28" t="n">
         <v>0</v>
       </c>
@@ -1121,20 +920,12 @@
       <c r="A29" t="n">
         <v>2048</v>
       </c>
-      <c r="B29" t="inlineStr"/>
       <c r="C29" t="n">
         <v>0</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
       </c>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
       <c r="L29" t="n">
         <v>0</v>
       </c>
@@ -1143,20 +934,12 @@
       <c r="A30" t="n">
         <v>2049</v>
       </c>
-      <c r="B30" t="inlineStr"/>
       <c r="C30" t="n">
         <v>0</v>
       </c>
       <c r="D30" t="n">
         <v>0</v>
       </c>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
       <c r="L30" t="n">
         <v>0</v>
       </c>
@@ -1165,20 +948,12 @@
       <c r="A31" t="n">
         <v>2050</v>
       </c>
-      <c r="B31" t="inlineStr"/>
       <c r="C31" t="n">
         <v>0</v>
       </c>
       <c r="D31" t="n">
         <v>0</v>
       </c>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
       <c r="L31" t="n">
         <v>0</v>
       </c>
@@ -1187,20 +962,12 @@
       <c r="A32" t="n">
         <v>2051</v>
       </c>
-      <c r="B32" t="inlineStr"/>
       <c r="C32" t="n">
         <v>0</v>
       </c>
       <c r="D32" t="n">
         <v>0</v>
       </c>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
       <c r="L32" t="n">
         <v>0</v>
       </c>
@@ -1209,20 +976,12 @@
       <c r="A33" t="n">
         <v>2052</v>
       </c>
-      <c r="B33" t="inlineStr"/>
       <c r="C33" t="n">
         <v>0</v>
       </c>
       <c r="D33" t="n">
         <v>0</v>
       </c>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
       <c r="L33" t="n">
         <v>0</v>
       </c>
@@ -1231,20 +990,12 @@
       <c r="A34" t="n">
         <v>2053</v>
       </c>
-      <c r="B34" t="inlineStr"/>
       <c r="C34" t="n">
         <v>0</v>
       </c>
       <c r="D34" t="n">
         <v>0</v>
       </c>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
       <c r="L34" t="n">
         <v>0</v>
       </c>
@@ -1253,20 +1004,12 @@
       <c r="A35" t="n">
         <v>2054</v>
       </c>
-      <c r="B35" t="inlineStr"/>
       <c r="C35" t="n">
         <v>0</v>
       </c>
       <c r="D35" t="n">
         <v>0</v>
       </c>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
       <c r="L35" t="n">
         <v>0</v>
       </c>
@@ -1275,20 +1018,12 @@
       <c r="A36" t="n">
         <v>2055</v>
       </c>
-      <c r="B36" t="inlineStr"/>
       <c r="C36" t="n">
         <v>0</v>
       </c>
       <c r="D36" t="n">
         <v>0</v>
       </c>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
       <c r="L36" t="n">
         <v>0</v>
       </c>
@@ -1373,22 +1108,15 @@
       <c r="A2" t="n">
         <v>2021</v>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
         <v>0</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
       <c r="I2" t="n">
         <v>4000</v>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="n">
         <v>0</v>
       </c>
@@ -1397,22 +1125,15 @@
       <c r="A3" t="n">
         <v>2022</v>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
         <v>4000</v>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="n">
         <v>0</v>
       </c>
@@ -1421,22 +1142,15 @@
       <c r="A4" t="n">
         <v>2023</v>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
         <v>0</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
         <v>4000</v>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
       <c r="L4" t="n">
         <v>0</v>
       </c>
@@ -1454,15 +1168,9 @@
       <c r="D5" t="n">
         <v>0</v>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
       <c r="J5" t="n">
         <v>12000</v>
       </c>
-      <c r="K5" t="inlineStr"/>
       <c r="L5" t="n">
         <v>0</v>
       </c>
@@ -1480,15 +1188,9 @@
       <c r="D6" t="n">
         <v>0</v>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
         <v>5000</v>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
       <c r="L6" t="n">
         <v>0</v>
       </c>
@@ -1506,13 +1208,6 @@
       <c r="D7" t="n">
         <v>0</v>
       </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
       <c r="L7" t="n">
         <v>4000</v>
       </c>
@@ -1530,13 +1225,6 @@
       <c r="D8" t="n">
         <v>0</v>
       </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
       <c r="L8" t="n">
         <v>4000</v>
       </c>
@@ -1554,13 +1242,6 @@
       <c r="D9" t="n">
         <v>0</v>
       </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
       <c r="L9" t="n">
         <v>0</v>
       </c>
@@ -1569,20 +1250,12 @@
       <c r="A10" t="n">
         <v>2029</v>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="n">
         <v>0</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
       </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
       <c r="L10" t="n">
         <v>0</v>
       </c>
@@ -1591,20 +1264,12 @@
       <c r="A11" t="n">
         <v>2030</v>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="n">
         <v>0</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
       </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
       <c r="L11" t="n">
         <v>0</v>
       </c>
@@ -1613,20 +1278,12 @@
       <c r="A12" t="n">
         <v>2031</v>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="n">
         <v>0</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
       </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
       <c r="L12" t="n">
         <v>0</v>
       </c>
@@ -1635,20 +1292,12 @@
       <c r="A13" t="n">
         <v>2032</v>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="n">
         <v>0</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
       </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
       <c r="L13" t="n">
         <v>0</v>
       </c>
@@ -1657,20 +1306,12 @@
       <c r="A14" t="n">
         <v>2033</v>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" t="n">
         <v>0</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
       </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
       <c r="L14" t="n">
         <v>0</v>
       </c>
@@ -1679,20 +1320,12 @@
       <c r="A15" t="n">
         <v>2034</v>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" t="n">
         <v>0</v>
       </c>
       <c r="D15" t="n">
         <v>0</v>
       </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
       <c r="L15" t="n">
         <v>0</v>
       </c>
@@ -1701,20 +1334,12 @@
       <c r="A16" t="n">
         <v>2035</v>
       </c>
-      <c r="B16" t="inlineStr"/>
       <c r="C16" t="n">
         <v>0</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
       </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
       <c r="L16" t="n">
         <v>0</v>
       </c>
@@ -1723,20 +1348,12 @@
       <c r="A17" t="n">
         <v>2036</v>
       </c>
-      <c r="B17" t="inlineStr"/>
       <c r="C17" t="n">
         <v>0</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
       </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
       <c r="L17" t="n">
         <v>0</v>
       </c>
@@ -1745,20 +1362,12 @@
       <c r="A18" t="n">
         <v>2037</v>
       </c>
-      <c r="B18" t="inlineStr"/>
       <c r="C18" t="n">
         <v>0</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
       </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
       <c r="L18" t="n">
         <v>0</v>
       </c>
@@ -1767,20 +1376,12 @@
       <c r="A19" t="n">
         <v>2038</v>
       </c>
-      <c r="B19" t="inlineStr"/>
       <c r="C19" t="n">
         <v>0</v>
       </c>
       <c r="D19" t="n">
         <v>0</v>
       </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
       <c r="L19" t="n">
         <v>0</v>
       </c>
@@ -1789,20 +1390,12 @@
       <c r="A20" t="n">
         <v>2039</v>
       </c>
-      <c r="B20" t="inlineStr"/>
       <c r="C20" t="n">
         <v>0</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
       </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
       <c r="L20" t="n">
         <v>0</v>
       </c>
@@ -1811,20 +1404,12 @@
       <c r="A21" t="n">
         <v>2040</v>
       </c>
-      <c r="B21" t="inlineStr"/>
       <c r="C21" t="n">
         <v>0</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
       </c>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
       <c r="L21" t="n">
         <v>0</v>
       </c>
@@ -1833,20 +1418,12 @@
       <c r="A22" t="n">
         <v>2041</v>
       </c>
-      <c r="B22" t="inlineStr"/>
       <c r="C22" t="n">
         <v>0</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
       </c>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
       <c r="L22" t="n">
         <v>0</v>
       </c>
@@ -1855,20 +1432,12 @@
       <c r="A23" t="n">
         <v>2042</v>
       </c>
-      <c r="B23" t="inlineStr"/>
       <c r="C23" t="n">
         <v>0</v>
       </c>
       <c r="D23" t="n">
         <v>0</v>
       </c>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
       <c r="L23" t="n">
         <v>0</v>
       </c>
@@ -1877,20 +1446,12 @@
       <c r="A24" t="n">
         <v>2043</v>
       </c>
-      <c r="B24" t="inlineStr"/>
       <c r="C24" t="n">
         <v>0</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
       </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
       <c r="L24" t="n">
         <v>0</v>
       </c>
@@ -1899,20 +1460,12 @@
       <c r="A25" t="n">
         <v>2044</v>
       </c>
-      <c r="B25" t="inlineStr"/>
       <c r="C25" t="n">
         <v>0</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
       </c>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
       <c r="L25" t="n">
         <v>0</v>
       </c>
@@ -1921,20 +1474,12 @@
       <c r="A26" t="n">
         <v>2045</v>
       </c>
-      <c r="B26" t="inlineStr"/>
       <c r="C26" t="n">
         <v>0</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
       </c>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
       <c r="L26" t="n">
         <v>0</v>
       </c>
@@ -1943,20 +1488,12 @@
       <c r="A27" t="n">
         <v>2046</v>
       </c>
-      <c r="B27" t="inlineStr"/>
       <c r="C27" t="n">
         <v>0</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
       </c>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
       <c r="L27" t="n">
         <v>0</v>
       </c>
@@ -1965,20 +1502,12 @@
       <c r="A28" t="n">
         <v>2047</v>
       </c>
-      <c r="B28" t="inlineStr"/>
       <c r="C28" t="n">
         <v>0</v>
       </c>
       <c r="D28" t="n">
         <v>0</v>
       </c>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
       <c r="L28" t="n">
         <v>0</v>
       </c>
@@ -1987,20 +1516,12 @@
       <c r="A29" t="n">
         <v>2048</v>
       </c>
-      <c r="B29" t="inlineStr"/>
       <c r="C29" t="n">
         <v>0</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
       </c>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
       <c r="L29" t="n">
         <v>0</v>
       </c>
@@ -2009,20 +1530,12 @@
       <c r="A30" t="n">
         <v>2049</v>
       </c>
-      <c r="B30" t="inlineStr"/>
       <c r="C30" t="n">
         <v>0</v>
       </c>
       <c r="D30" t="n">
         <v>0</v>
       </c>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
       <c r="L30" t="n">
         <v>0</v>
       </c>
@@ -2031,20 +1544,12 @@
       <c r="A31" t="n">
         <v>2050</v>
       </c>
-      <c r="B31" t="inlineStr"/>
       <c r="C31" t="n">
         <v>0</v>
       </c>
       <c r="D31" t="n">
         <v>0</v>
       </c>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
       <c r="L31" t="n">
         <v>0</v>
       </c>
@@ -2053,20 +1558,12 @@
       <c r="A32" t="n">
         <v>2051</v>
       </c>
-      <c r="B32" t="inlineStr"/>
       <c r="C32" t="n">
         <v>0</v>
       </c>
       <c r="D32" t="n">
         <v>0</v>
       </c>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
       <c r="L32" t="n">
         <v>0</v>
       </c>
@@ -2075,20 +1572,12 @@
       <c r="A33" t="n">
         <v>2052</v>
       </c>
-      <c r="B33" t="inlineStr"/>
       <c r="C33" t="n">
         <v>0</v>
       </c>
       <c r="D33" t="n">
         <v>0</v>
       </c>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
       <c r="L33" t="n">
         <v>0</v>
       </c>
@@ -2097,20 +1586,12 @@
       <c r="A34" t="n">
         <v>2053</v>
       </c>
-      <c r="B34" t="inlineStr"/>
       <c r="C34" t="n">
         <v>0</v>
       </c>
       <c r="D34" t="n">
         <v>0</v>
       </c>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
       <c r="L34" t="n">
         <v>0</v>
       </c>
@@ -2119,20 +1600,12 @@
       <c r="A35" t="n">
         <v>2054</v>
       </c>
-      <c r="B35" t="inlineStr"/>
       <c r="C35" t="n">
         <v>0</v>
       </c>
       <c r="D35" t="n">
         <v>0</v>
       </c>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
       <c r="L35" t="n">
         <v>0</v>
       </c>
@@ -2141,20 +1614,12 @@
       <c r="A36" t="n">
         <v>2055</v>
       </c>
-      <c r="B36" t="inlineStr"/>
       <c r="C36" t="n">
         <v>0</v>
       </c>
       <c r="D36" t="n">
         <v>0</v>
       </c>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
       <c r="L36" t="n">
         <v>0</v>
       </c>
@@ -2163,20 +1628,12 @@
       <c r="A37" t="n">
         <v>2056</v>
       </c>
-      <c r="B37" t="inlineStr"/>
       <c r="C37" t="n">
         <v>0</v>
       </c>
       <c r="D37" t="n">
         <v>0</v>
       </c>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
       <c r="L37" t="n">
         <v>0</v>
       </c>
@@ -2185,20 +1642,12 @@
       <c r="A38" t="n">
         <v>2057</v>
       </c>
-      <c r="B38" t="inlineStr"/>
       <c r="C38" t="n">
         <v>0</v>
       </c>
       <c r="D38" t="n">
         <v>0</v>
       </c>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
       <c r="L38" t="n">
         <v>0</v>
       </c>
@@ -2207,20 +1656,12 @@
       <c r="A39" t="n">
         <v>2058</v>
       </c>
-      <c r="B39" t="inlineStr"/>
       <c r="C39" t="n">
         <v>0</v>
       </c>
       <c r="D39" t="n">
         <v>0</v>
       </c>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
       <c r="L39" t="n">
         <v>0</v>
       </c>
@@ -2388,7 +1829,7 @@
         <v>750000</v>
       </c>
       <c r="G2" t="n">
-        <v>3.5</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
[feat] Add QCD capabilities per issue #137
</commit_message>
<xml_diff>
--- a/examples/HFP_alex+jamie.xlsx
+++ b/examples/HFP_alex+jamie.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alex" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jamie" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debts" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fixed Assets" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Alex" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Jamie" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Debts" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Fixed Assets" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,16 +20,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -428,66 +416,71 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:M36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>year</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>anticipated wages</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>other inc</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>net inv</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>taxable ctrb</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>401k ctrb</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Roth 401k ctrb</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>IRA ctrb</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Roth IRA ctrb</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Roth conv</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>QCD</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
         <is>
           <t>big-ticket items</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>HSA ctrb</t>
         </is>
@@ -497,16 +490,26 @@
       <c r="A2" t="n">
         <v>2021</v>
       </c>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
         <v>0</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
         <v>6500</v>
       </c>
-      <c r="L2" t="n">
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -514,16 +517,26 @@
       <c r="A3" t="n">
         <v>2022</v>
       </c>
+      <c r="B3" t="inlineStr"/>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
         <v>6500</v>
       </c>
-      <c r="L3" t="n">
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -531,16 +544,26 @@
       <c r="A4" t="n">
         <v>2023</v>
       </c>
+      <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
         <v>0</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
         <v>7000</v>
       </c>
-      <c r="L4" t="n">
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -557,10 +580,19 @@
       <c r="D5" t="n">
         <v>0</v>
       </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
         <v>7000</v>
       </c>
-      <c r="L5" t="n">
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -577,13 +609,21 @@
       <c r="D6" t="n">
         <v>0</v>
       </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
         <v>7000</v>
       </c>
+      <c r="I6" t="inlineStr"/>
       <c r="J6" t="n">
         <v>20000</v>
       </c>
-      <c r="L6" t="n">
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -600,10 +640,19 @@
       <c r="D7" t="n">
         <v>0</v>
       </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
         <v>15000</v>
       </c>
-      <c r="L7" t="n">
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="n">
         <v>4000</v>
       </c>
     </row>
@@ -620,10 +669,19 @@
       <c r="D8" t="n">
         <v>0</v>
       </c>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
         <v>15000</v>
       </c>
-      <c r="L8" t="n">
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="n">
         <v>4000</v>
       </c>
     </row>
@@ -640,10 +698,19 @@
       <c r="D9" t="n">
         <v>0</v>
       </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
       <c r="J9" t="n">
         <v>50000</v>
       </c>
-      <c r="L9" t="n">
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -651,16 +718,26 @@
       <c r="A10" t="n">
         <v>2029</v>
       </c>
+      <c r="B10" t="inlineStr"/>
       <c r="C10" t="n">
         <v>0</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
       </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
       <c r="J10" t="n">
         <v>50000</v>
       </c>
-      <c r="L10" t="n">
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -668,13 +745,24 @@
       <c r="A11" t="n">
         <v>2030</v>
       </c>
+      <c r="B11" t="inlineStr"/>
       <c r="C11" t="n">
         <v>0</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
       </c>
-      <c r="L11" t="n">
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -682,13 +770,24 @@
       <c r="A12" t="n">
         <v>2031</v>
       </c>
+      <c r="B12" t="inlineStr"/>
       <c r="C12" t="n">
         <v>0</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
       </c>
-      <c r="L12" t="n">
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="n">
         <v>0</v>
       </c>
     </row>
@@ -696,13 +795,24 @@
       <c r="A13" t="n">
         <v>2032</v>
       </c>
+      <c r="B13" t="inlineStr"/>
       <c r="C13" t="n">
         <v>0</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
       </c>
-      <c r="L13" t="n">
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="n">
         <v>0</v>
       </c>
     </row>
@@ -710,13 +820,24 @@
       <c r="A14" t="n">
         <v>2033</v>
       </c>
+      <c r="B14" t="inlineStr"/>
       <c r="C14" t="n">
         <v>0</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
       </c>
-      <c r="L14" t="n">
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -724,13 +845,24 @@
       <c r="A15" t="n">
         <v>2034</v>
       </c>
+      <c r="B15" t="inlineStr"/>
       <c r="C15" t="n">
         <v>0</v>
       </c>
       <c r="D15" t="n">
         <v>0</v>
       </c>
-      <c r="L15" t="n">
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="n">
         <v>0</v>
       </c>
     </row>
@@ -738,13 +870,24 @@
       <c r="A16" t="n">
         <v>2035</v>
       </c>
+      <c r="B16" t="inlineStr"/>
       <c r="C16" t="n">
         <v>0</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
       </c>
-      <c r="L16" t="n">
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="n">
         <v>0</v>
       </c>
     </row>
@@ -752,13 +895,24 @@
       <c r="A17" t="n">
         <v>2036</v>
       </c>
+      <c r="B17" t="inlineStr"/>
       <c r="C17" t="n">
         <v>0</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
       </c>
-      <c r="L17" t="n">
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="n">
         <v>0</v>
       </c>
     </row>
@@ -766,13 +920,24 @@
       <c r="A18" t="n">
         <v>2037</v>
       </c>
+      <c r="B18" t="inlineStr"/>
       <c r="C18" t="n">
         <v>0</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
       </c>
-      <c r="L18" t="n">
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="n">
         <v>0</v>
       </c>
     </row>
@@ -780,13 +945,24 @@
       <c r="A19" t="n">
         <v>2038</v>
       </c>
+      <c r="B19" t="inlineStr"/>
       <c r="C19" t="n">
         <v>0</v>
       </c>
       <c r="D19" t="n">
         <v>0</v>
       </c>
-      <c r="L19" t="n">
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -794,13 +970,24 @@
       <c r="A20" t="n">
         <v>2039</v>
       </c>
+      <c r="B20" t="inlineStr"/>
       <c r="C20" t="n">
         <v>0</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
       </c>
-      <c r="L20" t="n">
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="n">
         <v>0</v>
       </c>
     </row>
@@ -808,13 +995,24 @@
       <c r="A21" t="n">
         <v>2040</v>
       </c>
+      <c r="B21" t="inlineStr"/>
       <c r="C21" t="n">
         <v>0</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
       </c>
-      <c r="L21" t="n">
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="n">
         <v>0</v>
       </c>
     </row>
@@ -822,13 +1020,24 @@
       <c r="A22" t="n">
         <v>2041</v>
       </c>
+      <c r="B22" t="inlineStr"/>
       <c r="C22" t="n">
         <v>0</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
       </c>
-      <c r="L22" t="n">
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="n">
         <v>0</v>
       </c>
     </row>
@@ -836,13 +1045,24 @@
       <c r="A23" t="n">
         <v>2042</v>
       </c>
+      <c r="B23" t="inlineStr"/>
       <c r="C23" t="n">
         <v>0</v>
       </c>
       <c r="D23" t="n">
         <v>0</v>
       </c>
-      <c r="L23" t="n">
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="n">
         <v>0</v>
       </c>
     </row>
@@ -850,13 +1070,24 @@
       <c r="A24" t="n">
         <v>2043</v>
       </c>
+      <c r="B24" t="inlineStr"/>
       <c r="C24" t="n">
         <v>0</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
       </c>
-      <c r="L24" t="n">
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="n">
         <v>0</v>
       </c>
     </row>
@@ -864,13 +1095,24 @@
       <c r="A25" t="n">
         <v>2044</v>
       </c>
+      <c r="B25" t="inlineStr"/>
       <c r="C25" t="n">
         <v>0</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
       </c>
-      <c r="L25" t="n">
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="n">
         <v>0</v>
       </c>
     </row>
@@ -878,13 +1120,24 @@
       <c r="A26" t="n">
         <v>2045</v>
       </c>
+      <c r="B26" t="inlineStr"/>
       <c r="C26" t="n">
         <v>0</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
       </c>
-      <c r="L26" t="n">
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="n">
         <v>0</v>
       </c>
     </row>
@@ -892,13 +1145,24 @@
       <c r="A27" t="n">
         <v>2046</v>
       </c>
+      <c r="B27" t="inlineStr"/>
       <c r="C27" t="n">
         <v>0</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
       </c>
-      <c r="L27" t="n">
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="n">
         <v>0</v>
       </c>
     </row>
@@ -906,13 +1170,24 @@
       <c r="A28" t="n">
         <v>2047</v>
       </c>
+      <c r="B28" t="inlineStr"/>
       <c r="C28" t="n">
         <v>0</v>
       </c>
       <c r="D28" t="n">
         <v>0</v>
       </c>
-      <c r="L28" t="n">
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="n">
         <v>0</v>
       </c>
     </row>
@@ -920,13 +1195,24 @@
       <c r="A29" t="n">
         <v>2048</v>
       </c>
+      <c r="B29" t="inlineStr"/>
       <c r="C29" t="n">
         <v>0</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
       </c>
-      <c r="L29" t="n">
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="n">
         <v>0</v>
       </c>
     </row>
@@ -934,13 +1220,24 @@
       <c r="A30" t="n">
         <v>2049</v>
       </c>
+      <c r="B30" t="inlineStr"/>
       <c r="C30" t="n">
         <v>0</v>
       </c>
       <c r="D30" t="n">
         <v>0</v>
       </c>
-      <c r="L30" t="n">
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="n">
         <v>0</v>
       </c>
     </row>
@@ -948,13 +1245,24 @@
       <c r="A31" t="n">
         <v>2050</v>
       </c>
+      <c r="B31" t="inlineStr"/>
       <c r="C31" t="n">
         <v>0</v>
       </c>
       <c r="D31" t="n">
         <v>0</v>
       </c>
-      <c r="L31" t="n">
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -962,13 +1270,24 @@
       <c r="A32" t="n">
         <v>2051</v>
       </c>
+      <c r="B32" t="inlineStr"/>
       <c r="C32" t="n">
         <v>0</v>
       </c>
       <c r="D32" t="n">
         <v>0</v>
       </c>
-      <c r="L32" t="n">
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="n">
         <v>0</v>
       </c>
     </row>
@@ -976,13 +1295,24 @@
       <c r="A33" t="n">
         <v>2052</v>
       </c>
+      <c r="B33" t="inlineStr"/>
       <c r="C33" t="n">
         <v>0</v>
       </c>
       <c r="D33" t="n">
         <v>0</v>
       </c>
-      <c r="L33" t="n">
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="n">
         <v>0</v>
       </c>
     </row>
@@ -990,13 +1320,24 @@
       <c r="A34" t="n">
         <v>2053</v>
       </c>
+      <c r="B34" t="inlineStr"/>
       <c r="C34" t="n">
         <v>0</v>
       </c>
       <c r="D34" t="n">
         <v>0</v>
       </c>
-      <c r="L34" t="n">
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1004,13 +1345,24 @@
       <c r="A35" t="n">
         <v>2054</v>
       </c>
+      <c r="B35" t="inlineStr"/>
       <c r="C35" t="n">
         <v>0</v>
       </c>
       <c r="D35" t="n">
         <v>0</v>
       </c>
-      <c r="L35" t="n">
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1018,13 +1370,24 @@
       <c r="A36" t="n">
         <v>2055</v>
       </c>
+      <c r="B36" t="inlineStr"/>
       <c r="C36" t="n">
         <v>0</v>
       </c>
       <c r="D36" t="n">
         <v>0</v>
       </c>
-      <c r="L36" t="n">
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1039,66 +1402,71 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L39"/>
+  <dimension ref="A1:M39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>year</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>anticipated wages</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>other inc</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>net inv</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>taxable ctrb</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>401k ctrb</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Roth 401k ctrb</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>IRA ctrb</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Roth IRA ctrb</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Roth conv</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>QCD</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
         <is>
           <t>big-ticket items</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>HSA ctrb</t>
         </is>
@@ -1108,16 +1476,26 @@
       <c r="A2" t="n">
         <v>2021</v>
       </c>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
         <v>0</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
       <c r="I2" t="n">
         <v>4000</v>
       </c>
-      <c r="L2" t="n">
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1125,16 +1503,26 @@
       <c r="A3" t="n">
         <v>2022</v>
       </c>
+      <c r="B3" t="inlineStr"/>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
         <v>4000</v>
       </c>
-      <c r="L3" t="n">
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1142,16 +1530,26 @@
       <c r="A4" t="n">
         <v>2023</v>
       </c>
+      <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
         <v>0</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
         <v>4000</v>
       </c>
-      <c r="L4" t="n">
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1168,10 +1566,19 @@
       <c r="D5" t="n">
         <v>0</v>
       </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
       <c r="J5" t="n">
         <v>12000</v>
       </c>
-      <c r="L5" t="n">
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1188,10 +1595,19 @@
       <c r="D6" t="n">
         <v>0</v>
       </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
         <v>5000</v>
       </c>
-      <c r="L6" t="n">
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1208,7 +1624,17 @@
       <c r="D7" t="n">
         <v>0</v>
       </c>
-      <c r="L7" t="n">
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="n">
         <v>4000</v>
       </c>
     </row>
@@ -1225,7 +1651,17 @@
       <c r="D8" t="n">
         <v>0</v>
       </c>
-      <c r="L8" t="n">
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="n">
         <v>4000</v>
       </c>
     </row>
@@ -1242,7 +1678,17 @@
       <c r="D9" t="n">
         <v>0</v>
       </c>
-      <c r="L9" t="n">
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1250,13 +1696,24 @@
       <c r="A10" t="n">
         <v>2029</v>
       </c>
+      <c r="B10" t="inlineStr"/>
       <c r="C10" t="n">
         <v>0</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
       </c>
-      <c r="L10" t="n">
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1264,13 +1721,24 @@
       <c r="A11" t="n">
         <v>2030</v>
       </c>
+      <c r="B11" t="inlineStr"/>
       <c r="C11" t="n">
         <v>0</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
       </c>
-      <c r="L11" t="n">
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1278,13 +1746,24 @@
       <c r="A12" t="n">
         <v>2031</v>
       </c>
+      <c r="B12" t="inlineStr"/>
       <c r="C12" t="n">
         <v>0</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
       </c>
-      <c r="L12" t="n">
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1292,13 +1771,24 @@
       <c r="A13" t="n">
         <v>2032</v>
       </c>
+      <c r="B13" t="inlineStr"/>
       <c r="C13" t="n">
         <v>0</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
       </c>
-      <c r="L13" t="n">
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1306,13 +1796,24 @@
       <c r="A14" t="n">
         <v>2033</v>
       </c>
+      <c r="B14" t="inlineStr"/>
       <c r="C14" t="n">
         <v>0</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
       </c>
-      <c r="L14" t="n">
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1320,13 +1821,24 @@
       <c r="A15" t="n">
         <v>2034</v>
       </c>
+      <c r="B15" t="inlineStr"/>
       <c r="C15" t="n">
         <v>0</v>
       </c>
       <c r="D15" t="n">
         <v>0</v>
       </c>
-      <c r="L15" t="n">
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1334,13 +1846,24 @@
       <c r="A16" t="n">
         <v>2035</v>
       </c>
+      <c r="B16" t="inlineStr"/>
       <c r="C16" t="n">
         <v>0</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
       </c>
-      <c r="L16" t="n">
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1348,13 +1871,24 @@
       <c r="A17" t="n">
         <v>2036</v>
       </c>
+      <c r="B17" t="inlineStr"/>
       <c r="C17" t="n">
         <v>0</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
       </c>
-      <c r="L17" t="n">
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1362,13 +1896,24 @@
       <c r="A18" t="n">
         <v>2037</v>
       </c>
+      <c r="B18" t="inlineStr"/>
       <c r="C18" t="n">
         <v>0</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
       </c>
-      <c r="L18" t="n">
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1376,13 +1921,24 @@
       <c r="A19" t="n">
         <v>2038</v>
       </c>
+      <c r="B19" t="inlineStr"/>
       <c r="C19" t="n">
         <v>0</v>
       </c>
       <c r="D19" t="n">
         <v>0</v>
       </c>
-      <c r="L19" t="n">
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1390,13 +1946,24 @@
       <c r="A20" t="n">
         <v>2039</v>
       </c>
+      <c r="B20" t="inlineStr"/>
       <c r="C20" t="n">
         <v>0</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
       </c>
-      <c r="L20" t="n">
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1404,13 +1971,24 @@
       <c r="A21" t="n">
         <v>2040</v>
       </c>
+      <c r="B21" t="inlineStr"/>
       <c r="C21" t="n">
         <v>0</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
       </c>
-      <c r="L21" t="n">
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1418,13 +1996,24 @@
       <c r="A22" t="n">
         <v>2041</v>
       </c>
+      <c r="B22" t="inlineStr"/>
       <c r="C22" t="n">
         <v>0</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
       </c>
-      <c r="L22" t="n">
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1432,13 +2021,24 @@
       <c r="A23" t="n">
         <v>2042</v>
       </c>
+      <c r="B23" t="inlineStr"/>
       <c r="C23" t="n">
         <v>0</v>
       </c>
       <c r="D23" t="n">
         <v>0</v>
       </c>
-      <c r="L23" t="n">
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1446,13 +2046,24 @@
       <c r="A24" t="n">
         <v>2043</v>
       </c>
+      <c r="B24" t="inlineStr"/>
       <c r="C24" t="n">
         <v>0</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
       </c>
-      <c r="L24" t="n">
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1460,13 +2071,24 @@
       <c r="A25" t="n">
         <v>2044</v>
       </c>
+      <c r="B25" t="inlineStr"/>
       <c r="C25" t="n">
         <v>0</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
       </c>
-      <c r="L25" t="n">
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1474,13 +2096,24 @@
       <c r="A26" t="n">
         <v>2045</v>
       </c>
+      <c r="B26" t="inlineStr"/>
       <c r="C26" t="n">
         <v>0</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
       </c>
-      <c r="L26" t="n">
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1488,13 +2121,24 @@
       <c r="A27" t="n">
         <v>2046</v>
       </c>
+      <c r="B27" t="inlineStr"/>
       <c r="C27" t="n">
         <v>0</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
       </c>
-      <c r="L27" t="n">
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1502,13 +2146,24 @@
       <c r="A28" t="n">
         <v>2047</v>
       </c>
+      <c r="B28" t="inlineStr"/>
       <c r="C28" t="n">
         <v>0</v>
       </c>
       <c r="D28" t="n">
         <v>0</v>
       </c>
-      <c r="L28" t="n">
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1516,13 +2171,24 @@
       <c r="A29" t="n">
         <v>2048</v>
       </c>
+      <c r="B29" t="inlineStr"/>
       <c r="C29" t="n">
         <v>0</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
       </c>
-      <c r="L29" t="n">
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1530,13 +2196,24 @@
       <c r="A30" t="n">
         <v>2049</v>
       </c>
+      <c r="B30" t="inlineStr"/>
       <c r="C30" t="n">
         <v>0</v>
       </c>
       <c r="D30" t="n">
         <v>0</v>
       </c>
-      <c r="L30" t="n">
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1544,13 +2221,24 @@
       <c r="A31" t="n">
         <v>2050</v>
       </c>
+      <c r="B31" t="inlineStr"/>
       <c r="C31" t="n">
         <v>0</v>
       </c>
       <c r="D31" t="n">
         <v>0</v>
       </c>
-      <c r="L31" t="n">
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1558,13 +2246,24 @@
       <c r="A32" t="n">
         <v>2051</v>
       </c>
+      <c r="B32" t="inlineStr"/>
       <c r="C32" t="n">
         <v>0</v>
       </c>
       <c r="D32" t="n">
         <v>0</v>
       </c>
-      <c r="L32" t="n">
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1572,13 +2271,24 @@
       <c r="A33" t="n">
         <v>2052</v>
       </c>
+      <c r="B33" t="inlineStr"/>
       <c r="C33" t="n">
         <v>0</v>
       </c>
       <c r="D33" t="n">
         <v>0</v>
       </c>
-      <c r="L33" t="n">
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1586,13 +2296,24 @@
       <c r="A34" t="n">
         <v>2053</v>
       </c>
+      <c r="B34" t="inlineStr"/>
       <c r="C34" t="n">
         <v>0</v>
       </c>
       <c r="D34" t="n">
         <v>0</v>
       </c>
-      <c r="L34" t="n">
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1600,13 +2321,24 @@
       <c r="A35" t="n">
         <v>2054</v>
       </c>
+      <c r="B35" t="inlineStr"/>
       <c r="C35" t="n">
         <v>0</v>
       </c>
       <c r="D35" t="n">
         <v>0</v>
       </c>
-      <c r="L35" t="n">
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1614,13 +2346,24 @@
       <c r="A36" t="n">
         <v>2055</v>
       </c>
+      <c r="B36" t="inlineStr"/>
       <c r="C36" t="n">
         <v>0</v>
       </c>
       <c r="D36" t="n">
         <v>0</v>
       </c>
-      <c r="L36" t="n">
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1628,13 +2371,24 @@
       <c r="A37" t="n">
         <v>2056</v>
       </c>
+      <c r="B37" t="inlineStr"/>
       <c r="C37" t="n">
         <v>0</v>
       </c>
       <c r="D37" t="n">
         <v>0</v>
       </c>
-      <c r="L37" t="n">
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="n">
+        <v>0</v>
+      </c>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1642,13 +2396,24 @@
       <c r="A38" t="n">
         <v>2057</v>
       </c>
+      <c r="B38" t="inlineStr"/>
       <c r="C38" t="n">
         <v>0</v>
       </c>
       <c r="D38" t="n">
         <v>0</v>
       </c>
-      <c r="L38" t="n">
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="n">
+        <v>0</v>
+      </c>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1656,13 +2421,24 @@
       <c r="A39" t="n">
         <v>2058</v>
       </c>
+      <c r="B39" t="inlineStr"/>
       <c r="C39" t="n">
         <v>0</v>
       </c>
       <c r="D39" t="n">
         <v>0</v>
       </c>
-      <c r="L39" t="n">
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="n">
+        <v>0</v>
+      </c>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1681,37 +2457,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>year</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>term</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>amount</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>rate</t>
         </is>
@@ -1759,47 +2535,47 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>year</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>basis</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>value</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>rate</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>yod</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>commission</t>
         </is>

</xml_diff>